<commit_message>
campo landing page criado
</commit_message>
<xml_diff>
--- a/novos_leads.xlsx
+++ b/novos_leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,11 @@
           <t>unidadeform</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Landing Page ou Formulário de Origem</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -469,6 +474,11 @@
           <t>Medicina Lorena</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Medicina - Formulário Meta</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -496,6 +506,11 @@
           <t>Canaã</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ARQ - Formulário Meta</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -521,6 +536,11 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>Canaã</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>AGR - Formulário Meta</t>
         </is>
       </c>
     </row>

</xml_diff>